<commit_message>
[docs] 요구사항분석서 v1.4.2 반영 (CR-006)
- SFR-167 AI 일지 정리 Should → Could (D-125)
- SFR-092 iOS 무음 모드 안내 명시 (SFR-130 참조와 맞춤)
- SFR-168 만료 배너 규칙 명확화, SFR-146 중복 시나리오 삭제 (D-126)
- INR-002 카카오 내비 SDK 승인 기록
- 정리: SER-011·016의 SFR-150 참조 제거, SFR-113 근거 SER-007, DAR-014·COR 7건 확정, ID 파란색 규칙·조건부 서식 삭제

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/요구사항분석서.xlsx
+++ b/docs/요구사항분석서.xlsx
@@ -1354,7 +1354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I143"/>
+  <dimension ref="A1:I145"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="34" min="1" max="1"/>
@@ -8056,16 +8056,105 @@
         </is>
       </c>
     </row>
+    <row r="144" ht="70" customHeight="1" s="35">
+      <c r="A144" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D-125</t>
+        </is>
+      </c>
+      <c r="B144" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SFR-167 / D-111</t>
+        </is>
+      </c>
+      <c r="C144" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AI 일지 정리 우선순위</t>
+        </is>
+      </c>
+      <c r="D144" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">① Should 유지 ② Could</t>
+        </is>
+      </c>
+      <c r="E144" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">② Could (일정 여유가 있으면 S7)</t>
+        </is>
+      </c>
+      <c r="F144" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">일지 초안·내보내기(Must)로 핵심 효과는 충족, 8주 일정 여유 확보</t>
+        </is>
+      </c>
+      <c r="G144" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-27</t>
+        </is>
+      </c>
+      <c r="H144" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">확정</t>
+        </is>
+      </c>
+      <c r="I144" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v1.4.2 / CR-006</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="70" customHeight="1" s="35">
+      <c r="A145" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D-126</t>
+        </is>
+      </c>
+      <c r="B145" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SFR-168, 146</t>
+        </is>
+      </c>
+      <c r="C145" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">라이선스 만료 배너 표시 규칙</t>
+        </is>
+      </c>
+      <c r="D145" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">① 30·7·1일 당일만 ② 30일 전부터 매번 + 단계별 강조</t>
+        </is>
+      </c>
+      <c r="E145" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">② 30일 전부터 근무 시작마다, 7일 이하 빨간색, 1일 이하 닫기 불가</t>
+        </is>
+      </c>
+      <c r="F145" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'전부터' 해석이 갈림, 만료 직전에 놓치는 것 방지</t>
+        </is>
+      </c>
+      <c r="G145" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-27</t>
+        </is>
+      </c>
+      <c r="H145" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">확정</t>
+        </is>
+      </c>
+      <c r="I145" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v1.4.2 / CR-006</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I118"/>
   <conditionalFormatting sqref="A2:I500">
     <cfRule type="expression" rank="0" priority="2" equalAverage="0" aboveAverage="0" dxfId="13" text="" percent="0" bottom="0">
       <formula>$H2="미결"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A500">
-    <cfRule type="expression" rank="0" priority="3" equalAverage="0" aboveAverage="0" dxfId="6" text="" percent="0" bottom="0">
-      <formula>ISNUMBER(SEARCH("v0.115",$I2))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -8086,7 +8175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="34" min="1" max="1"/>
@@ -8461,6 +8550,58 @@
       <c r="J7" s="65" t="inlineStr">
         <is>
           <t>v1.4.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="110" customHeight="1" s="35">
+      <c r="A8" s="65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR-006</t>
+        </is>
+      </c>
+      <c r="B8" s="65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-27</t>
+        </is>
+      </c>
+      <c r="C8" s="66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">백강욱</t>
+        </is>
+      </c>
+      <c r="D8" s="65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SFR-167·092·168·146·113, INR-002, SER-011·016, DAR-014, COR-004·007·008·009·012·013·014, 00_표지 사용 규칙 8</t>
+        </is>
+      </c>
+      <c r="E8" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">① AI 일지 정리(SFR-167) Should → Could ② iOS 무음 모드 안내를 SFR-092에 명시(SFR-130 참조와 맞춤) ③ 만료 배너 규칙 명확화: 30일 전부터 근무 시작마다, 7일 이하 빨간색, 1일 이하 닫기 불가 / SFR-146의 배너 시나리오 삭제 ④ 카카오 내비 SDK 사용 승인 완료 기록(INR-002) ⑤ 정리: 삭제된 SFR-150 참조 제거(SER-011·016), SFR-113 14시간 근거를 SER-007로, DAR-014 확정(3년), 남은 제약사항 '초안' 7건 확정, ID 칸 파란색 규칙 삭제(사용 규칙 8·조건부 서식)</t>
+        </is>
+      </c>
+      <c r="F8" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">일정 여유 확보, 참조 불일치·해석이 갈리는 문구 정리, 외부 승인 완료, 베이스라인 이후 남은 '초안' 상태 정리</t>
+        </is>
+      </c>
+      <c r="G8" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">화면: 병원 웹 만료 배너 색·닫기 버튼, 앱 iOS 알림 권한 안내 1줄 / API·DB: 변경 없음 / 일정: 감소(SFR-167 Could)</t>
+        </is>
+      </c>
+      <c r="H8" s="66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">승인</t>
+        </is>
+      </c>
+      <c r="I8" s="65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-27</t>
+        </is>
+      </c>
+      <c r="J8" s="65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v1.4.2</t>
         </is>
       </c>
     </row>
@@ -11273,7 +11414,7 @@
       </c>
       <c r="B6" s="42" t="inlineStr">
         <is>
-          <t>v1.4.1</t>
+          <t xml:space="preserve">v1.4.2</t>
         </is>
       </c>
       <c r="C6" s="46" t="n"/>
@@ -12120,6 +12261,16 @@
           <t>2</t>
         </is>
       </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">백강욱</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v1.4.2 (2026-10-27): CR-006 승인 — AI 일지 정리 Could로(D-125), iOS 무음 모드 안내 SFR-092 명시, 만료 배너 규칙 명확화·SFR-146 중복 삭제(D-126), 카카오 내비 SDK 승인 반영, 정리(SFR-150 참조 제거, SFR-113 근거, DAR-014·제약 7건 확정, 파란색 규칙 삭제)</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="35">
       <c r="A49" s="41" t="inlineStr">
@@ -12256,7 +12407,7 @@
       </c>
       <c r="B60" s="42" t="inlineStr">
         <is>
-          <t>ID 칸이 파란색 = v0.115에서 신규·수정된 행. 비고에 무엇이 바뀌었는지 적혀 있다</t>
+          <t xml:space="preserve">변경 이력은 비고 칸의 [vX 신규]·[vX 수정] 태그로 확인한다 (ID 칸 파란색 표시는 v1.4.2에서 없앰)</t>
         </is>
       </c>
       <c r="C60" s="46" t="n"/>
@@ -13478,12 +13629,12 @@
       </c>
       <c r="F3" s="41" t="inlineStr">
         <is>
-          <t>첫 실행 시, 시스템은 위치 → 전화 → 알림 순서로 권한을 요청하고(iOS는 전화 권한이 없어 위치 → 알림), 권한마다 필요한 이유를 한 문장으로 표시해야 한다. 위치 권한은 필수이므로, 거부하면 '위치 권한이 있어야 사용할 수 있어요' 안내와 설정으로 이동 버튼을 보여주고 허용할 때까지 다음 단계로 넘어가지 않는다(SFR-041). 알림 권한을 거부하면 '병원 승인을 소리·진동으로만 알 수 있어요'를 안내한다. (알림: SFR-130) 위치는 '앱 사용 중 허용'만 요청하고 백그라운드 위치 권한은 요청하지 않는다(SFR-079). 카메라 권한은 첫 실행 때 묻지 않고 공무원증 촬영(SFR-017)·QR 스캔(SFR-113) 때 요청한다.</t>
+          <t xml:space="preserve">첫 실행 시, 시스템은 위치 → 전화 → 알림 순서로 권한을 요청하고(iOS는 전화 권한이 없어 위치 → 알림), 권한마다 필요한 이유를 한 문장으로 표시해야 한다. 위치 권한은 필수이므로, 거부하면 '위치 권한이 있어야 사용할 수 있어요' 안내와 설정으로 이동 버튼을 보여주고 허용할 때까지 다음 단계로 넘어가지 않는다(SFR-041). 알림 권한을 거부하면 '병원 승인을 소리·진동으로만 알 수 있어요'를 안내한다. (알림: SFR-130) iOS에서는 알림 권한 이유 문장에 '무음 모드에서는 소리 없이 진동으로만 알려요'를 함께 표시한다. 위치는 '앱 사용 중 허용'만 요청하고 백그라운드 위치 권한은 요청하지 않는다(SFR-079). 카메라 권한은 첫 실행 때 묻지 않고 공무원증 촬영(SFR-017)·QR 스캔(SFR-113) 때 요청한다.</t>
         </is>
       </c>
       <c r="G3" s="42" t="inlineStr">
         <is>
-          <t>Given Android 폰에서 앱을 처음 실행함
+          <t xml:space="preserve">Given Android 폰에서 앱을 처음 실행함
 When 권한 요청 단계로 넘어간다
 Then 위치 → 전화 → 알림 순서로 권한 요청이 표시된다
 And 각 요청 앞에 필요한 이유 한 문장이 표시된다
@@ -13495,7 +13646,10 @@
 Then '병원 승인을 소리·진동으로만 알 수 있어요' 안내가 표시되고 다음 단계로 넘어간다
 Given iPhone에서 앱을 처음 실행함
 When 권한 요청 단계로 넘어간다
-Then 위치 → 알림 순서로만 표시되고 전화 권한 요청은 없다</t>
+Then 위치 → 알림 순서로만 표시되고 전화 권한 요청은 없다
+Given iPhone에서 앱을 처음 실행함
+When 알림 권한 요청 단계로 넘어간다
+Then 알림 권한 이유 문장에 '무음 모드에서는 소리 없이 진동으로만 알려요'가 함께 표시된다</t>
         </is>
       </c>
       <c r="H3" s="48" t="inlineStr">
@@ -13540,12 +13694,12 @@
       </c>
       <c r="P3" s="48" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t xml:space="preserve">2026-10-27</t>
         </is>
       </c>
       <c r="Q3" s="42" t="inlineStr">
         <is>
-          <t>[v0.92 신규]  / [v0.96 수정] Should→Must (Must 요구사항의 선행, C-15) / [v0.94] 인수 기준 추가 / [v0.105 수정] 알림 권한 추가 (D-63) / [v0.107 수정] 카메라 권한 시점 (D-73) / [v0.108 수정] 백그라운드 위치 권한 제거, 위치 거부해도 나머지 권한 계속 (검토) / [v0.111 수정] iOS 권한 순서(위치 → 알림) (D-97) / [v1.1 수정] 위치 권한 거부 시 진행 막음 (CR-001)</t>
+          <t xml:space="preserve">[v0.92 신규]  / [v0.96 수정] Should→Must (Must 요구사항의 선행, C-15) / [v0.94] 인수 기준 추가 / [v0.105 수정] 알림 권한 추가 (D-63) / [v0.107 수정] 카메라 권한 시점 (D-73) / [v0.108 수정] 백그라운드 위치 권한 제거, 위치 거부해도 나머지 권한 계속 (검토) / [v0.111 수정] iOS 권한 순서(위치 → 알림) (D-97) / [v1.1 수정] 위치 권한 거부 시 진행 막음 (CR-001) / [v1.4.2 수정] iOS 무음 모드 안내 명시 — SFR-130 참조와 맞춤 (CR-006)</t>
         </is>
       </c>
       <c r="R3" s="41" t="n"/>
@@ -14509,7 +14663,7 @@
       </c>
       <c r="F14" s="41" t="inlineStr">
         <is>
-          <t>시스템은 로그인한 구급대원이 근무를 시작할 때 팀을 만들거나 참여하게 해야 한다. 팀은 구급차 1대에 탄 대원(최대 4명)이며, 한 명이 팀을 만들면 4자리 코드와 QR을 표시하고 다른 대원은 코드 입력 또는 QR 스캔으로 참여한다(목록에서 초대하는 방식: SFR-159, 그 뒤로 코드·QR은 목록에 없는 대원용 예비 수단). 팀원은 각자 '운전'·'처치' 역할을 고르며 '운전'은 팀에 최대 1명이다. 참여자가 아직 없어도 팀을 만든 대원은 바로 환자 정보 입력으로 넘어갈 수 있다. '근무 종료'나 로그아웃을 하면 그 대원만 팀에서 빠지고, 마지막 1명이 빠지면 팀이 해제된다. 진행 중 이송 건이 있으면 빠지기 전에 '진행 중 이송 1건이 있어요'를 경고하고, 마지막 1명이면 이송 건을 '취소'(사유 '근무 종료')로 끝낼지 확인받는다. 승인된 계정만 팀에 참여할 수 있다. 근무 시작 후 14시간(초안)이 지나고 진행 중 이송이 없으면 자동으로 근무 종료(팀에서 빠짐)하고, 로그아웃(SFR-070)과 같게 처리해 다음 실행 때 로그인 화면을 보여준다. 대원이 직접 누른 근무 종료도 로그아웃과 같다.</t>
+          <t xml:space="preserve">시스템은 로그인한 구급대원이 근무를 시작할 때 팀을 만들거나 참여하게 해야 한다. 팀은 구급차 1대에 탄 대원(최대 4명)이며, 한 명이 팀을 만들면 4자리 코드와 QR을 표시하고 다른 대원은 코드 입력 또는 QR 스캔으로 참여한다(목록에서 초대하는 방식: SFR-159, 그 뒤로 코드·QR은 목록에 없는 대원용 예비 수단). 팀원은 각자 '운전'·'처치' 역할을 고르며 '운전'은 팀에 최대 1명이다. 참여자가 아직 없어도 팀을 만든 대원은 바로 환자 정보 입력으로 넘어갈 수 있다. '근무 종료'나 로그아웃을 하면 그 대원만 팀에서 빠지고, 마지막 1명이 빠지면 팀이 해제된다. 진행 중 이송 건이 있으면 빠지기 전에 '진행 중 이송 1건이 있어요'를 경고하고, 마지막 1명이면 이송 건을 '취소'(사유 '근무 종료')로 끝낼지 확인받는다. 승인된 계정만 팀에 참여할 수 있다. 근무 시작 후 14시간(SER-007)이 지나고 진행 중 이송이 없으면 자동으로 근무 종료(팀에서 빠짐)하고, 로그아웃(SFR-070)과 같게 처리해 다음 실행 때 로그인 화면을 보여준다. 대원이 직접 누른 근무 종료도 로그아웃과 같다.</t>
         </is>
       </c>
       <c r="G14" s="42" t="inlineStr">
@@ -14576,12 +14730,12 @@
       </c>
       <c r="P14" s="48" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t xml:space="preserve">2026-10-27</t>
         </is>
       </c>
       <c r="Q14" s="42" t="inlineStr">
         <is>
-          <t>[v0.98 신규] 9/29 회의 / [v0.100 수정] CPR 2대 출동 시 합류, 최대 6명 (D-47) / [v0.103 수정] 차량 1대=팀 1개, 최대 4명, 운전 1명, 근무 시작 시 필수 → Must·S2 (D-61) / [v0.107 수정] 코드·QR → 관할 소방서 대원 목록에서 초대·수락, 동명이인 구분, 코드·QR은 예비 (D-64) / [v0.108 수정] S2는 코드·QR로 맺기만, 목록 초대는 SFR-159(S5)로 분리, 근무 종료는 본인만 빠짐 (D-85, D-94) / [v0.110 수정] 개발 충돌 점검 (D-96) / [v1.4 수정] 근무 종료(직접·자동) = 로그아웃 (CR-004, D-110)</t>
+          <t xml:space="preserve">[v0.98 신규] 9/29 회의 / [v0.100 수정] CPR 2대 출동 시 합류, 최대 6명 (D-47) / [v0.103 수정] 차량 1대=팀 1개, 최대 4명, 운전 1명, 근무 시작 시 필수 → Must·S2 (D-61) / [v0.107 수정] 코드·QR → 관할 소방서 대원 목록에서 초대·수락, 동명이인 구분, 코드·QR은 예비 (D-64) / [v0.108 수정] S2는 코드·QR로 맺기만, 목록 초대는 SFR-159(S5)로 분리, 근무 종료는 본인만 빠짐 (D-85, D-94) / [v0.110 수정] 개발 충돌 점검 (D-96) / [v1.4 수정] 근무 종료(직접·자동) = 로그아웃 (CR-004, D-110) / [v1.4.2 수정] 14시간 근거를 확정값 SER-007로 (CR-006)</t>
         </is>
       </c>
       <c r="R14" s="42" t="inlineStr">
@@ -24097,16 +24251,13 @@
       </c>
       <c r="G115" s="42" t="inlineStr">
         <is>
-          <t>Given A병원 PC 2대가 등록되어 있음
+          <t xml:space="preserve">Given A병원 PC 2대가 등록되어 있음
 When 관리자가 사유 '병원 탈퇴'로 A병원 키를 '폐기'한다
 Then 2대 모두 병원 웹이 막히고, 새 키는 만들어지지 않는다
 Given A병원 PC 3대가 등록되어 있음
 When 관리자가 사유 '키 유출 의심'으로 A병원 키를 '재발급'한다
 Then 3대 모두 병원 웹이 막히고 키 입력 화면이 표시된다
 And 새 키가 한 번 전체 표시되고 작업 이력에 사유와 함께 기록된다
-Given A병원 키 만료까지 20일 남음
-When A병원 PC에서 병원 웹을 연다
-Then 상단에 '라이선스 키가 20일 뒤 만료돼요'가 표시된다
 Given A병원 키가 만료됨
 When 등록된 PC에서 병원 웹을 연다
 Then 병원 웹이 막히고 '라이선스 키가 만료됐어요, 관리자에게 문의하세요'가 표시된다</t>
@@ -24154,12 +24305,12 @@
       </c>
       <c r="P115" s="48" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t xml:space="preserve">2026-10-27</t>
         </is>
       </c>
       <c r="Q115" s="42" t="inlineStr">
         <is>
-          <t>[v0.107 신규] 9/30 회의·PM 결정 / [v0.108 수정] Must → Should (핵심 흐름이 기대지 않음, D-80) / [v1.4.1 수정] 만료 배너는 SFR-168로 일원화 (CR-005)</t>
+          <t xml:space="preserve">[v0.107 신규] 9/30 회의·PM 결정 / [v0.108 수정] Must → Should (핵심 흐름이 기대지 않음, D-80) / [v1.4.1 수정] 만료 배너는 SFR-168로 일원화 (CR-005) / [v1.4.2 수정] 만료 배너 시나리오 삭제 — SFR-168에서만 검증 (CR-006)</t>
         </is>
       </c>
       <c r="R115" s="42" t="inlineStr">
@@ -28878,7 +29029,7 @@
       </c>
       <c r="H168" s="48" t="inlineStr">
         <is>
-          <t>Should</t>
+          <t xml:space="preserve">Could</t>
         </is>
       </c>
       <c r="I168" s="48" t="inlineStr">
@@ -28913,17 +29064,17 @@
       </c>
       <c r="O168" s="42" t="inlineStr">
         <is>
-          <t>D-111</t>
+          <t xml:space="preserve">D-111, D-125</t>
         </is>
       </c>
       <c r="P168" s="48" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t xml:space="preserve">2026-10-27</t>
         </is>
       </c>
       <c r="Q168" s="42" t="inlineStr">
         <is>
-          <t>[v1.4 신규] (CR-004)</t>
+          <t xml:space="preserve">[v1.4 신규] (CR-004) / [v1.4.2 수정] Should → Could, 일정 여유가 있으면 구현 (CR-006, D-125)</t>
         </is>
       </c>
       <c r="R168" s="41" t="inlineStr">
@@ -28960,14 +29111,23 @@
       </c>
       <c r="F169" s="41" t="inlineStr">
         <is>
-          <t>병원 라이선스 키 만료 30일·7일·1일 전부터, 시스템은 병원 웹 상단에 '라이선스 키가 ○일 뒤 만료돼요 · 관리자에게 재발급을 요청하세요' 배너를 표시해야 한다. 배너는 닫아도 다음 근무 시작 때 다시 보인다.</t>
+          <t xml:space="preserve">병원 라이선스 키 만료 30일 전부터, 시스템은 병원 웹에서 근무를 시작할 때마다 상단에 '라이선스 키가 ○일 뒤 만료돼요 · 관리자에게 재발급을 요청하세요' 배너를 표시해야 한다. 남은 기간이 7일 이하면 빨간색으로 강조하고, 1일 이하면 닫을 수 없게 한다. 그 전에는 배너를 닫아도 다음 근무 시작 때 다시 보인다. 관리자 알림(만료 30일·7일·1일 전 1번씩)은 SFR-100을 따른다.</t>
         </is>
       </c>
       <c r="G169" s="42" t="inlineStr">
         <is>
-          <t>Given A병원 키 만료까지 7일
+          <t xml:space="preserve">Given A병원 키 만료까지 20일
 When 담당자가 근무 시작을 한다
-Then 상단에 '라이선스 키가 7일 뒤 만료돼요' 배너가 표시된다
+Then 상단에 기본 색 배너 '라이선스 키가 20일 뒤 만료돼요'가 표시된다
+Given 같은 상태에서 배너를 닫음
+When 다음 근무 시작을 한다
+Then 배너가 다시 표시된다
+Given A병원 키 만료까지 7일
+When 근무 시작을 한다
+Then 배너가 빨간색으로 표시된다
+Given A병원 키 만료까지 1일
+When 배너를 닫으려 한다
+Then 닫기 버튼이 없어 닫히지 않는다
 Given A병원 키 만료까지 40일
 When 근무 시작을 한다
 Then 배너가 표시되지 않는다</t>
@@ -29010,17 +29170,17 @@
       </c>
       <c r="O169" s="42" t="inlineStr">
         <is>
-          <t>D-116</t>
+          <t xml:space="preserve">D-116, D-126</t>
         </is>
       </c>
       <c r="P169" s="48" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t xml:space="preserve">2026-10-27</t>
         </is>
       </c>
       <c r="Q169" s="42" t="inlineStr">
         <is>
-          <t>[v1.4 신규] (CR-004)</t>
+          <t xml:space="preserve">[v1.4 신규] (CR-004) / [v1.4.2 수정] 30일 전부터 매 근무 시작, 7일 이하 빨간색, 1일 이하 닫기 불가 (CR-006, D-126)</t>
         </is>
       </c>
       <c r="R169" s="41" t="inlineStr">
@@ -29031,11 +29191,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:R162"/>
-  <conditionalFormatting sqref="A2:A500">
-    <cfRule type="expression" rank="0" priority="2" equalAverage="0" aboveAverage="0" dxfId="6" text="" percent="0" bottom="0">
-      <formula>ISNUMBER(SEARCH("v0.115",$Q2))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="A2:Q500">
     <cfRule type="expression" rank="0" priority="3" equalAverage="0" aboveAverage="0" dxfId="7" text="" percent="0" bottom="0">
       <formula>$N2="삭제"</formula>
@@ -30522,7 +30677,7 @@
       </c>
       <c r="G28" s="42" t="inlineStr">
         <is>
-          <t>SFR-018, 082, 116, 150, 152</t>
+          <t xml:space="preserve">SFR-018, 082, 116, 152</t>
         </is>
       </c>
       <c r="H28" s="49" t="inlineStr">
@@ -30537,7 +30692,7 @@
       </c>
       <c r="J28" s="42" t="inlineStr">
         <is>
-          <t>[v0.92 신규] 관리자 계정 보호 / [v0.102 수정] 병원 웹 포함 (D-54) / [v0.107 수정] 병원은 라이선스 키 입력 기준, 앱 PIN·OTP 추가 (D-70, D-74, D-75) / [v1.4 수정] 앱 PIN 삭제 (D-110)</t>
+          <t xml:space="preserve">[v0.92 신규] 관리자 계정 보호 / [v0.102 수정] 병원 웹 포함 (D-54) / [v0.107 수정] 병원은 라이선스 키 입력 기준, 앱 PIN·OTP 추가 (D-70, D-74, D-75) / [v1.4 수정] 앱 PIN 삭제 (D-110) / [v1.4.2 수정] 삭제된 SFR-150 참조 제거 (CR-006)</t>
         </is>
       </c>
     </row>
@@ -31317,7 +31472,7 @@
       </c>
       <c r="J43" s="42" t="inlineStr">
         <is>
-          <t>[v0.99 수정] TMAP → 카카오 (D-26) / [v0.103 수정] 요청용·예비 추천용 산출 방식 구분 (오류 12), 비상업 사용 권한 신청 필요 (ASM-04, 오류 24) / [v1.2 수정] 10km 밖 추정값, 이동 중은 내비 SDK 값, 호출 수 감시 (CR-002, D-106, ASM-12) / [v1.3 수정] 이동 중 외부 내비 분기 삭제, 관련 SFR에 121 추가 (CR-003)</t>
+          <t xml:space="preserve">[v0.99 수정] TMAP → 카카오 (D-26) / [v0.103 수정] 요청용·예비 추천용 산출 방식 구분 (오류 12), 비상업 사용 권한 신청 필요 (ASM-04, 오류 24) / [v1.2 수정] 10km 밖 추정값, 이동 중은 내비 SDK 값, 호출 수 감시 (CR-002, D-106, ASM-12) / [v1.3 수정] 이동 중 외부 내비 분기 삭제, 관련 SFR에 121 추가 (CR-003) / [v1.4.2] 카카오 내비 SDK 사용 승인 완료 (CR-006)</t>
         </is>
       </c>
     </row>
@@ -31718,7 +31873,7 @@
       </c>
       <c r="G51" s="42" t="inlineStr">
         <is>
-          <t>SFR-018, 070, 150, 151</t>
+          <t xml:space="preserve">SFR-018, 070, 151</t>
         </is>
       </c>
       <c r="H51" s="49" t="inlineStr">
@@ -31733,7 +31888,7 @@
       </c>
       <c r="J51" s="42" t="inlineStr">
         <is>
-          <t>[v0.110 신규] D-96 / [v1.3 수정] 요청마다 계정 상태 확인 — 접근 토큰 유효시간(15분) 동안 정지 계정이 통과하는 문제 (CR-003, D-107) / [v1.4 수정] PIN 5회 실패 조건 삭제 (D-110)</t>
+          <t xml:space="preserve">[v0.110 신규] D-96 / [v1.3 수정] 요청마다 계정 상태 확인 — 접근 토큰 유효시간(15분) 동안 정지 계정이 통과하는 문제 (CR-003, D-107) / [v1.4 수정] PIN 5회 실패 조건 삭제 (D-110) / [v1.4.2 수정] 삭제된 SFR-150 참조 제거 (CR-006)</t>
         </is>
       </c>
     </row>
@@ -31916,7 +32071,7 @@
       </c>
       <c r="E55" s="49" t="inlineStr">
         <is>
-          <t>3년 (초안, 기관 확인)</t>
+          <t xml:space="preserve">3년</t>
         </is>
       </c>
       <c r="F55" s="41" t="inlineStr">
@@ -31936,12 +32091,12 @@
       </c>
       <c r="I55" s="49" t="inlineStr">
         <is>
-          <t>초안</t>
+          <t xml:space="preserve">확정</t>
         </is>
       </c>
       <c r="J55" s="42" t="inlineStr">
         <is>
-          <t>[v1.4 신규] 향후 구급대원용 내비 개발 데이터 (CR-004, D-113)</t>
+          <t xml:space="preserve">[v1.4 신규] 향후 구급대원용 내비 개발 데이터 (CR-004, D-113) / [v1.4.2 수정] 확정 — 기관 확인 결과가 다르면 CR (CR-006)</t>
         </is>
       </c>
     </row>
@@ -32259,11 +32414,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:J51"/>
-  <conditionalFormatting sqref="A2:A500">
-    <cfRule type="expression" rank="0" priority="2" equalAverage="0" aboveAverage="0" dxfId="6" text="" percent="0" bottom="0">
-      <formula>ISNUMBER(SEARCH("v0.115",$J2))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="A2:J500">
     <cfRule type="expression" rank="0" priority="3" equalAverage="0" aboveAverage="0" dxfId="7" text="" percent="0" bottom="0">
       <formula>$I2="삭제"</formula>
@@ -32472,12 +32622,12 @@
       </c>
       <c r="E6" s="49" t="inlineStr">
         <is>
-          <t>초안</t>
+          <t xml:space="preserve">확정</t>
         </is>
       </c>
       <c r="F6" s="42" t="inlineStr">
         <is>
-          <t>[v0.92 신규] 테스트 중 운영 데이터 훼손 방지 / [v0.103 수정] 시연 환경을 운영과 분리 (오류 2)</t>
+          <t xml:space="preserve">[v0.92 신규] 테스트 중 운영 데이터 훼손 방지 / [v0.103 수정] 시연 환경을 운영과 분리 (오류 2) / [v1.4.2] 초안 → 확정 (CR-006)</t>
         </is>
       </c>
     </row>
@@ -32504,12 +32654,12 @@
       </c>
       <c r="E7" s="49" t="inlineStr">
         <is>
-          <t>초안</t>
+          <t xml:space="preserve">확정</t>
         </is>
       </c>
       <c r="F7" s="42" t="inlineStr">
         <is>
-          <t>[v0.96 신규] SFR-017 '등록된 코드'의 출처, 검토 지적 반영 / [v0.107 수정] 관리자 가입 메뉴 없음 명시 (D-75) / [v0.108 수정] 목록 초대가 S5로 이동 (D-85)</t>
+          <t xml:space="preserve">[v0.96 신규] SFR-017 '등록된 코드'의 출처, 검토 지적 반영 / [v0.107 수정] 관리자 가입 메뉴 없음 명시 (D-75) / [v0.108 수정] 목록 초대가 S5로 이동 (D-85) / [v1.4.2] 초안 → 확정 (CR-006)</t>
         </is>
       </c>
     </row>
@@ -32600,12 +32750,12 @@
       </c>
       <c r="E10" s="49" t="inlineStr">
         <is>
-          <t>초안</t>
+          <t xml:space="preserve">확정</t>
         </is>
       </c>
       <c r="F10" s="42" t="inlineStr">
         <is>
-          <t>[v0.100 신규] 결정 D-51 / [v0.111 수정] iOS는 APNs 경유 (D-97) / [v1.4 수정] 푸시 구조 명시 (D-119)</t>
+          <t xml:space="preserve">[v0.100 신규] 결정 D-51 / [v0.111 수정] iOS는 APNs 경유 (D-97) / [v1.4 수정] 푸시 구조 명시 (D-119) / [v1.4.2] 초안 → 확정 (CR-006)</t>
         </is>
       </c>
     </row>
@@ -32632,12 +32782,12 @@
       </c>
       <c r="E11" s="49" t="inlineStr">
         <is>
-          <t>초안</t>
+          <t xml:space="preserve">확정</t>
         </is>
       </c>
       <c r="F11" s="42" t="inlineStr">
         <is>
-          <t>[v0.98 신규] 결정 D-27 / [v0.107 수정] 웹만 (D-72) / [v0.108 수정] 탭 절전 방지 안내 (D-93) / [v1.4 수정] 관리자 분리 배포 (D-117)</t>
+          <t xml:space="preserve">[v0.98 신규] 결정 D-27 / [v0.107 수정] 웹만 (D-72) / [v0.108 수정] 탭 절전 방지 안내 (D-93) / [v1.4 수정] 관리자 분리 배포 (D-117) / [v1.4.2] 초안 → 확정 (CR-006)</t>
         </is>
       </c>
     </row>
@@ -32728,12 +32878,12 @@
       </c>
       <c r="E14" s="49" t="inlineStr">
         <is>
-          <t>초안</t>
+          <t xml:space="preserve">확정</t>
         </is>
       </c>
       <c r="F14" s="42" t="inlineStr">
         <is>
-          <t>[v0.107 신규] 결정 D-70</t>
+          <t xml:space="preserve">[v0.107 신규] 결정 D-70 / [v1.4.2] 초안 → 확정 (CR-006)</t>
         </is>
       </c>
     </row>
@@ -32760,12 +32910,12 @@
       </c>
       <c r="E15" s="49" t="inlineStr">
         <is>
-          <t>초안</t>
+          <t xml:space="preserve">확정</t>
         </is>
       </c>
       <c r="F15" s="42" t="inlineStr">
         <is>
-          <t>[v0.107 신규] 결정 D-70</t>
+          <t xml:space="preserve">[v0.107 신규] 결정 D-70 / [v1.4.2] 초안 → 확정 (CR-006)</t>
         </is>
       </c>
     </row>
@@ -32792,12 +32942,12 @@
       </c>
       <c r="E16" s="49" t="inlineStr">
         <is>
-          <t>초안</t>
+          <t xml:space="preserve">확정</t>
         </is>
       </c>
       <c r="F16" s="42" t="inlineStr">
         <is>
-          <t>[v0.111 신규] D-97 / [v1.4 수정] 앱 잠금 삭제 (D-110)</t>
+          <t xml:space="preserve">[v0.111 신규] D-97 / [v1.4 수정] 앱 잠금 삭제 (D-110) / [v1.4.2] 초안 → 확정 (CR-006)</t>
         </is>
       </c>
     </row>
@@ -33160,11 +33310,6 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A3:A17">
-    <cfRule type="expression" rank="0" priority="2" equalAverage="0" aboveAverage="0" dxfId="6" text="" percent="0" bottom="0">
-      <formula>ISNUMBER(SEARCH("v0.115",$F2))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>